<commit_message>
feat: add project docs and utility scripts for PA replacement requirements
This commit adds:
1. NGFW3.7 one-stop manual PDF and requirement comparison Excel
2. 5 utility scripts to process requirement docs and excel:
   - dump_req58.py: extract 58 requirements to text file
   - dump_matrix111.py: export function comparison matrix
   - build_topsec_pages.py: index topsec manual HTML pages
   - build_pa_pages.py: extract text and bookmarks from PA PDF docs
   - p2_trial.py: fill trial data into comparison excel
   - p2_apply.py: batch add functions and build requirement mapping sheet
3. Generated output text files from the scripts
</commit_message>
<xml_diff>
--- a/对比工作底稿.xlsx
+++ b/对比工作底稿.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待验证移交清单" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资料登记表" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="范围基线" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求映射" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,8 +64,14 @@
       <color rgb="001F2937"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +96,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,6 +150,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -217,102 +236,6 @@
 </file>
 
 <file path=xl/drawings/drawing_wm1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="6800000" y="6400000"/>
@@ -456,102 +379,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing_wm3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/drawings/drawing_wm4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
@@ -648,7 +475,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing_wm5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing_wm6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="6800000" y="6400000"/>
@@ -3224,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4524,34 +4351,66 @@
       <c r="L44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>IPS</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>特征库规模与更新</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="inlineStr"/>
-      <c r="G45" s="5" t="inlineStr"/>
-      <c r="H45" s="5" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
-      <c r="J45" s="5" t="inlineStr"/>
-      <c r="K45" s="5" t="inlineStr"/>
-      <c r="L45" s="5" t="inlineStr"/>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>入侵防御模块内置规则集（预定义+自定义规则+白名单），规则库经升级中心在线/离线更新；特征条数官方文档未公布，P3 从产品彩页/规格页核实</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>需订阅授权</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Threat Prevention 订阅；Vulnerability Protection（防漏洞）+Anti-Spyware（防间谍软件）两配置文件；特征库经 Dynamic Updates 更新</t>
+        </is>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>试填校验行</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>天融信CHM:入侵防御[topic10/200-202]+升级中心[topic61]；PA:Web帮助&gt;安全配置文件&gt;Vulnerability/Anti-Spyware+Device&gt;Dynamic Updates</t>
+        </is>
+      </c>
+      <c r="K45" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="inlineStr">
+        <is>
+          <t>P2试填</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -5408,34 +5267,66 @@
       <c r="L74" s="6" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+      <c r="A75" s="11" t="inlineStr">
         <is>
           <t>67</t>
         </is>
       </c>
-      <c r="B75" s="5" t="inlineStr">
+      <c r="B75" s="11" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C75" s="11" t="inlineStr">
         <is>
           <t>IPSec VPN</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D75" s="11" t="inlineStr">
         <is>
           <t>IKEv1/IKEv2 支持</t>
         </is>
       </c>
-      <c r="E75" s="5" t="inlineStr"/>
-      <c r="F75" s="5" t="inlineStr"/>
-      <c r="G75" s="5" t="inlineStr"/>
-      <c r="H75" s="5" t="inlineStr"/>
-      <c r="I75" s="5" t="inlineStr"/>
-      <c r="J75" s="5" t="inlineStr"/>
-      <c r="K75" s="5" t="inlineStr"/>
-      <c r="L75" s="5" t="inlineStr"/>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t>IPSecVPN 章含 IKE 配置（静态隧道/手工隧道两形态），IKEv1/IKEv2 支持细节 P3 读正文确认</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="H75" s="11" t="inlineStr">
+        <is>
+          <t>IKE Gateways 网关对象显式支持 IKEv1/IKEv2（IKEv2 优先/仅 IKEv2 模式），IKE Crypto 独立配置套件</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>试填校验行</t>
+        </is>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>天融信CHM:IPSecVPN[ipsec.html/静态隧道topic4]；PA:Web帮助&gt;Network Profiles&gt;IKE Gateways/IKE Crypto</t>
+        </is>
+      </c>
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L75" s="11" t="inlineStr">
+        <is>
+          <t>P2试填</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -6030,34 +5921,66 @@
       <c r="L95" s="5" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="8" t="inlineStr">
         <is>
           <t>87</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="8" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C96" s="8" t="inlineStr">
         <is>
           <t>HA</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
+      <c r="D96" s="8" t="inlineStr">
         <is>
           <t>主备/主主模式</t>
         </is>
       </c>
-      <c r="E96" s="4" t="inlineStr"/>
-      <c r="F96" s="4" t="inlineStr"/>
-      <c r="G96" s="4" t="inlineStr"/>
-      <c r="H96" s="4" t="inlineStr"/>
-      <c r="I96" s="4" t="inlineStr"/>
-      <c r="J96" s="4" t="inlineStr"/>
-      <c r="K96" s="4" t="inlineStr"/>
-      <c r="L96" s="4" t="inlineStr"/>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>高可用模块（状态/配置/链路探测/链路备份），双机热备主备模式；双活经虚系统+集群实现（案例四），主主原生形态 P3 确认</t>
+        </is>
+      </c>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>Device&gt;High Availability：主动/被动与主动/主动两种模式均原生支持（配置同步+会话同步+路径监控）</t>
+        </is>
+      </c>
+      <c r="I96" s="8" t="inlineStr">
+        <is>
+          <t>试填校验行</t>
+        </is>
+      </c>
+      <c r="J96" s="8" t="inlineStr">
+        <is>
+          <t>天融信CHM:高可用[toc462734581]+案例一/案例四；PA:Web帮助&gt;Device&gt;High Availability(主动/主动配置)</t>
+        </is>
+      </c>
+      <c r="K96" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L96" s="8" t="inlineStr">
+        <is>
+          <t>P2试填</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -6822,6 +6745,1126 @@
       <c r="J122" s="4" t="inlineStr"/>
       <c r="K122" s="4" t="inlineStr"/>
       <c r="L122" s="4" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="n">
+        <v>112</v>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>路由</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>BFD 双向转发检测</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr"/>
+      <c r="F123" s="9" t="inlineStr"/>
+      <c r="G123" s="9" t="inlineStr"/>
+      <c r="H123" s="9" t="inlineStr"/>
+      <c r="I123" s="9" t="inlineStr"/>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:BFD章[bfd.html]；PA:Network Profiles&gt;BFD Profile</t>
+        </is>
+      </c>
+      <c r="K123" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L123" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="9" t="n">
+        <v>113</v>
+      </c>
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>路由</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>ECMP 等价多路径</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr"/>
+      <c r="F124" s="9" t="inlineStr"/>
+      <c r="G124" s="9" t="inlineStr"/>
+      <c r="H124" s="9" t="inlineStr"/>
+      <c r="I124" s="9" t="inlineStr"/>
+      <c r="J124" s="9" t="inlineStr">
+        <is>
+          <t>天融信:待验证(CHM未见专章)；PA:虚拟路由器&gt;ECMP</t>
+        </is>
+      </c>
+      <c r="K124" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L124" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="n">
+        <v>114</v>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>网络服务</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>DNS 代理与 DNS Doctoring</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr"/>
+      <c r="F125" s="9" t="inlineStr"/>
+      <c r="G125" s="9" t="inlineStr"/>
+      <c r="H125" s="9" t="inlineStr"/>
+      <c r="I125" s="9" t="inlineStr"/>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:DNS服务器/域名记录/DNS Doctoring；PA:Network&gt;DNS Proxy</t>
+        </is>
+      </c>
+      <c r="K125" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L125" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>二层网络</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>VXLAN（二层/三层网关）</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr"/>
+      <c r="F126" s="9" t="inlineStr"/>
+      <c r="G126" s="9" t="inlineStr"/>
+      <c r="H126" s="9" t="inlineStr"/>
+      <c r="I126" s="9" t="inlineStr"/>
+      <c r="J126" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:VXLAN章[vxlan.html]+配置实例；PA:11.1待核实</t>
+        </is>
+      </c>
+      <c r="K126" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L126" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="n">
+        <v>116</v>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>网络服务</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>MACsec 链路加密</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr"/>
+      <c r="F127" s="9" t="inlineStr"/>
+      <c r="G127" s="9" t="inlineStr"/>
+      <c r="H127" s="9" t="inlineStr"/>
+      <c r="I127" s="9" t="inlineStr"/>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>天融信:未见；PA:Network Profiles&gt;MACsec Profile(11.1)</t>
+        </is>
+      </c>
+      <c r="K127" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L127" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="9" t="n">
+        <v>117</v>
+      </c>
+      <c r="B128" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>网络服务</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>PPPoE 客户端接入</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="inlineStr"/>
+      <c r="F128" s="9" t="inlineStr"/>
+      <c r="G128" s="9" t="inlineStr"/>
+      <c r="H128" s="9" t="inlineStr"/>
+      <c r="I128" s="9" t="inlineStr"/>
+      <c r="J128" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:PPPoE章[pppoe.html]；PA:接口支持PPPoE</t>
+        </is>
+      </c>
+      <c r="K128" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L128" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="9" t="n">
+        <v>118</v>
+      </c>
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>IPv6</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>IPv6 过渡隧道（ISATAP/6to4/6in4）</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr"/>
+      <c r="F129" s="9" t="inlineStr"/>
+      <c r="G129" s="9" t="inlineStr"/>
+      <c r="H129" s="9" t="inlineStr"/>
+      <c r="I129" s="9" t="inlineStr"/>
+      <c r="J129" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:隧道章三协议专节；PA:待核实</t>
+        </is>
+      </c>
+      <c r="K129" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L129" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="9" t="n">
+        <v>119</v>
+      </c>
+      <c r="B130" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>负载均衡</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>服务器负载均衡 SLB</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr"/>
+      <c r="F130" s="9" t="inlineStr"/>
+      <c r="G130" s="9" t="inlineStr"/>
+      <c r="H130" s="9" t="inlineStr"/>
+      <c r="I130" s="9" t="inlineStr"/>
+      <c r="J130" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:资源管理&gt;负载均衡/服务器；PA:无内置(生态外置)</t>
+        </is>
+      </c>
+      <c r="K130" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L130" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>负载均衡</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>链路负载均衡 LLB</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr"/>
+      <c r="F131" s="9" t="inlineStr"/>
+      <c r="G131" s="9" t="inlineStr"/>
+      <c r="H131" s="9" t="inlineStr"/>
+      <c r="I131" s="9" t="inlineStr"/>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:链路负载均衡/链路池/本地链路；PA:无LLB(SD-WAN路径选择替代,实现路径不同)</t>
+        </is>
+      </c>
+      <c r="K131" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L131" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="9" t="n">
+        <v>121</v>
+      </c>
+      <c r="B132" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>识别技术</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>移动网络协议保护（GTP/SCTP/MNP）</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr"/>
+      <c r="F132" s="9" t="inlineStr"/>
+      <c r="G132" s="9" t="inlineStr"/>
+      <c r="H132" s="9" t="inlineStr"/>
+      <c r="I132" s="9" t="inlineStr"/>
+      <c r="J132" s="9" t="inlineStr">
+        <is>
+          <t>天融信:无；PA:MNP/SCTP Protection Profile(电信场景)</t>
+        </is>
+      </c>
+      <c r="K132" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L132" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="9" t="n">
+        <v>122</v>
+      </c>
+      <c r="B133" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>应用控制</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>网络数据包代理（NPBroker）</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr"/>
+      <c r="F133" s="9" t="inlineStr"/>
+      <c r="G133" s="9" t="inlineStr"/>
+      <c r="H133" s="9" t="inlineStr"/>
+      <c r="I133" s="9" t="inlineStr"/>
+      <c r="J133" s="9" t="inlineStr">
+        <is>
+          <t>天融信:无(端口镜像替代)；PA:Policies&gt;Network Packet Broker(11.1)</t>
+        </is>
+      </c>
+      <c r="K133" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L133" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="9" t="n">
+        <v>123</v>
+      </c>
+      <c r="B134" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>识别技术</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>IoT 设备识别与资产清单</t>
+        </is>
+      </c>
+      <c r="E134" s="9" t="inlineStr"/>
+      <c r="F134" s="9" t="inlineStr"/>
+      <c r="G134" s="9" t="inlineStr"/>
+      <c r="H134" s="9" t="inlineStr"/>
+      <c r="I134" s="9" t="inlineStr"/>
+      <c r="J134" s="9" t="inlineStr">
+        <is>
+          <t>天融信:资产发现(安全中心)；PA:IoT Security订阅+设备资产清单</t>
+        </is>
+      </c>
+      <c r="K134" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L134" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="9" t="n">
+        <v>124</v>
+      </c>
+      <c r="B135" s="9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>SSL 解密</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>解密流量镜像与解密排除</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr"/>
+      <c r="F135" s="9" t="inlineStr"/>
+      <c r="G135" s="9" t="inlineStr"/>
+      <c r="H135" s="9" t="inlineStr"/>
+      <c r="I135" s="9" t="inlineStr"/>
+      <c r="J135" s="9" t="inlineStr">
+        <is>
+          <t>天融信:SSL卸载策略[R58]；PA:解密镜像接口+SSL解密排除(11.1)</t>
+        </is>
+      </c>
+      <c r="K135" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L135" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B136" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>威胁检测</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>工控协议识别与防护</t>
+        </is>
+      </c>
+      <c r="E136" s="9" t="inlineStr"/>
+      <c r="F136" s="9" t="inlineStr"/>
+      <c r="G136" s="9" t="inlineStr"/>
+      <c r="H136" s="9" t="inlineStr"/>
+      <c r="I136" s="9" t="inlineStr"/>
+      <c r="J136" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:工业安全章(工控策略组/地址策略/值策略)；PA:无内置</t>
+        </is>
+      </c>
+      <c r="K136" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L136" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="n">
+        <v>126</v>
+      </c>
+      <c r="B137" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>威胁检测</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>数据库访问防护</t>
+        </is>
+      </c>
+      <c r="E137" s="9" t="inlineStr"/>
+      <c r="F137" s="9" t="inlineStr"/>
+      <c r="G137" s="9" t="inlineStr"/>
+      <c r="H137" s="9" t="inlineStr"/>
+      <c r="I137" s="9" t="inlineStr"/>
+      <c r="J137" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:数据库安全章(防护/自学习/基线/风险语句)；PA:无内置</t>
+        </is>
+      </c>
+      <c r="K137" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L137" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="n">
+        <v>127</v>
+      </c>
+      <c r="B138" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>威胁检测</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>弱口令检测</t>
+        </is>
+      </c>
+      <c r="E138" s="9" t="inlineStr"/>
+      <c r="F138" s="9" t="inlineStr"/>
+      <c r="G138" s="9" t="inlineStr"/>
+      <c r="H138" s="9" t="inlineStr"/>
+      <c r="I138" s="9" t="inlineStr"/>
+      <c r="J138" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:高级威胁防护&gt;弱口令[topic205]；PA:无直接对应</t>
+        </is>
+      </c>
+      <c r="K138" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L138" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="9" t="n">
+        <v>128</v>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>威胁检测</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>隧道检测（Tunnel Inspection）</t>
+        </is>
+      </c>
+      <c r="E139" s="9" t="inlineStr"/>
+      <c r="F139" s="9" t="inlineStr"/>
+      <c r="G139" s="9" t="inlineStr"/>
+      <c r="H139" s="9" t="inlineStr"/>
+      <c r="I139" s="9" t="inlineStr"/>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>天融信:IPS兼做；PA:独立策略类型(11.1)</t>
+        </is>
+      </c>
+      <c r="K139" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L139" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="9" t="n">
+        <v>129</v>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C140" s="9" t="inlineStr">
+        <is>
+          <t>组网</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>SD-WAN（路径选择/链路质量探测/流量分发）</t>
+        </is>
+      </c>
+      <c r="E140" s="9" t="inlineStr"/>
+      <c r="F140" s="9" t="inlineStr"/>
+      <c r="G140" s="9" t="inlineStr"/>
+      <c r="H140" s="9" t="inlineStr"/>
+      <c r="I140" s="9" t="inlineStr"/>
+      <c r="J140" s="9" t="inlineStr">
+        <is>
+          <t>天融信:无SD-WAN(LLB+策略路由部分实现)；PA:完整SD-WAN体系(策略/链路管理/接口)</t>
+        </is>
+      </c>
+      <c r="K140" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L140" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>SSL VPN</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>终端合规检查（HIP）</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr"/>
+      <c r="F141" s="9" t="inlineStr"/>
+      <c r="G141" s="9" t="inlineStr"/>
+      <c r="H141" s="9" t="inlineStr"/>
+      <c r="I141" s="9" t="inlineStr"/>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>天融信:无；PA:GlobalProtect HIP对象/配置文件/MDM</t>
+        </is>
+      </c>
+      <c r="K141" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L141" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="9" t="n">
+        <v>131</v>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C142" s="9" t="inlineStr">
+        <is>
+          <t>IPSec VPN</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>抗量子 VPN（PQ KEM）</t>
+        </is>
+      </c>
+      <c r="E142" s="9" t="inlineStr"/>
+      <c r="F142" s="9" t="inlineStr"/>
+      <c r="G142" s="9" t="inlineStr"/>
+      <c r="H142" s="9" t="inlineStr"/>
+      <c r="I142" s="9" t="inlineStr"/>
+      <c r="J142" s="9" t="inlineStr">
+        <is>
+          <t>天融信:无；PA:PAN-OS 12.1新增(HQ KEM算术套件)</t>
+        </is>
+      </c>
+      <c r="K142" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L142" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="9" t="n">
+        <v>132</v>
+      </c>
+      <c r="B143" s="9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>配置管理</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>策略优化器与宽泛策略分析</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr"/>
+      <c r="F143" s="9" t="inlineStr"/>
+      <c r="G143" s="9" t="inlineStr"/>
+      <c r="H143" s="9" t="inlineStr"/>
+      <c r="I143" s="9" t="inlineStr"/>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:策略分析及管理/宽泛策略分析；PA:Security Policy Optimizer+规则使用统计</t>
+        </is>
+      </c>
+      <c r="K143" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L143" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="n">
+        <v>133</v>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C144" s="9" t="inlineStr">
+        <is>
+          <t>密钥管理</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>HSM 硬件安全模块与主密钥</t>
+        </is>
+      </c>
+      <c r="E144" s="9" t="inlineStr"/>
+      <c r="F144" s="9" t="inlineStr"/>
+      <c r="G144" s="9" t="inlineStr"/>
+      <c r="H144" s="9" t="inlineStr"/>
+      <c r="I144" s="9" t="inlineStr"/>
+      <c r="J144" s="9" t="inlineStr">
+        <is>
+          <t>天融信:未见；PA:Device&gt;Setup&gt;HSM+Master Key</t>
+        </is>
+      </c>
+      <c r="K144" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L144" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="9" t="n">
+        <v>134</v>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>运维诊断</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>网络诊断与抓包</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr"/>
+      <c r="F145" s="9" t="inlineStr"/>
+      <c r="G145" s="9" t="inlineStr"/>
+      <c r="H145" s="9" t="inlineStr"/>
+      <c r="I145" s="9" t="inlineStr"/>
+      <c r="J145" s="9" t="inlineStr">
+        <is>
+          <t>天融信CHM:网络诊断/网络抓包；PA:Packet Capture+Ping/Traceroute</t>
+        </is>
+      </c>
+      <c r="K145" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L145" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C146" s="9" t="inlineStr">
+        <is>
+          <t>配置管理</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>配置锁与并发编辑控制</t>
+        </is>
+      </c>
+      <c r="E146" s="9" t="inlineStr"/>
+      <c r="F146" s="9" t="inlineStr"/>
+      <c r="G146" s="9" t="inlineStr"/>
+      <c r="H146" s="9" t="inlineStr"/>
+      <c r="I146" s="9" t="inlineStr"/>
+      <c r="J146" s="9" t="inlineStr">
+        <is>
+          <t>天融信:待验证(对应R25)；PA:Web界面锁定配置(11.1)</t>
+        </is>
+      </c>
+      <c r="K146" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L146" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="n">
+        <v>136</v>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>形态</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>5G 蜂窝接口</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr"/>
+      <c r="F147" s="9" t="inlineStr"/>
+      <c r="G147" s="9" t="inlineStr"/>
+      <c r="H147" s="9" t="inlineStr"/>
+      <c r="I147" s="9" t="inlineStr"/>
+      <c r="J147" s="9" t="inlineStr">
+        <is>
+          <t>天融信:待核实；PA:PA-415-5G+蜂窝接口(11.1)</t>
+        </is>
+      </c>
+      <c r="K147" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L147" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="9" t="n">
+        <v>137</v>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>接口</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>PoE 供电输出</t>
+        </is>
+      </c>
+      <c r="E148" s="9" t="inlineStr"/>
+      <c r="F148" s="9" t="inlineStr"/>
+      <c r="G148" s="9" t="inlineStr"/>
+      <c r="H148" s="9" t="inlineStr"/>
+      <c r="I148" s="9" t="inlineStr"/>
+      <c r="J148" s="9" t="inlineStr">
+        <is>
+          <t>天融信:未见；PA:PA-1400/PA-500 PoE(330W)</t>
+        </is>
+      </c>
+      <c r="K148" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L148" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="9" t="n">
+        <v>138</v>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>形态</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>工业加固型号</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr"/>
+      <c r="F149" s="9" t="inlineStr"/>
+      <c r="G149" s="9" t="inlineStr"/>
+      <c r="H149" s="9" t="inlineStr"/>
+      <c r="I149" s="9" t="inlineStr"/>
+      <c r="J149" s="9" t="inlineStr">
+        <is>
+          <t>天融信:工业防火墙产品线；PA:PA-400R系列</t>
+        </is>
+      </c>
+      <c r="K149" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L149" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="9" t="n">
+        <v>139</v>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>扩展</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>专用日志转发卡</t>
+        </is>
+      </c>
+      <c r="E150" s="9" t="inlineStr"/>
+      <c r="F150" s="9" t="inlineStr"/>
+      <c r="G150" s="9" t="inlineStr"/>
+      <c r="H150" s="9" t="inlineStr"/>
+      <c r="I150" s="9" t="inlineStr"/>
+      <c r="J150" s="9" t="inlineStr">
+        <is>
+          <t>天融信:无此形态(集中管理平台替代)；PA:Log Forwarding Card(PA-5400/7000)</t>
+        </is>
+      </c>
+      <c r="K150" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="L150" s="9" t="inlineStr">
+        <is>
+          <t>P2增补</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7156,7 +8199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8192,9 +9235,6 @@
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
     </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -8301,12 +9341,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>OS 平台 NGTOS（64位多核并行）；手册基线《NGFW一本通》文档编号 V3.2406.37098（©2025）；OS 具体版本号官网未公开，建议 400-777-0777 核实</t>
+          <t>系统版本 NGFW V3.7（CHM 文件名 NGFW3.7一本通.hhc，P2 确认）；OS 平台 NGTOS（64位多核并行）；手册文档编号 V3.2406.37098（©2025）；建议 400-777-0777 核实 V3.7 是否最新在售</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>本地 CHM《一本通》文档约定页 + 官网产品页，2026-08-15</t>
+          <t>CHM 目录文件名 + 手册文档约定页，2026-08-15</t>
         </is>
       </c>
     </row>
@@ -8487,4 +9527,1666 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>PA替代需求 58 条 → 功能对比矩阵功能点映射（P2 产出）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>运维 / 邮件告警 / 支持SMTPS协议发送邮件告警</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>完全支持映射 F84</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>邮件告警(SMTPS)属日志外发/告警子项</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>运维 / 第三方对接 / 支持对接FireMon</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>F83</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>FireMon 经 REST/XML API 对接配置管理</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>运维 / 第三方对接 / 支持对接Ansiable</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>F83</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Ansible 经 API+Playbook 对接</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>运维 / 第三方对接 / 支持restful api</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>F83</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>RESTful API 覆盖对象/策略/NAT/路由/接口</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 支持基于源IP过滤</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>日志过滤字段属日志能力</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 支持基于目的IP过滤</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 支持基于源端口过滤</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 支持基于目的端口过滤</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 连接日志支持记录会话开始时间</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>连接日志字段（会话开始时间）</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 连接日志支持记录会话结束时间</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>连接日志字段（会话结束时间）</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>运维 / 日志 / 连接日志支持记录会话结束原因</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>连接日志字段（结束原因）</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>运维 / 授权 / 授权平滑升级（开启模块和授权延长）</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>F91</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>授权平滑升级属授权管理</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持Facebook应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>港澳国际应用识别：识别库规模+覆盖度（R13 Facebook）</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>R14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持Youtube应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>R15</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持Twitter（X）应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Twitter(X)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持WhatsApp应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持TikTok应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>R18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持Zoom应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>R19</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持steam应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持Office365应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Office365（子应用识别 B27）</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>R21</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>应用控制 / 应用和协议识别控制 / 支持TeamView应用识别和控制</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>B24+B36</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>TeamViewer</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>R22</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>SSLVPN / 用户认证 / 支持双因子认证</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>E74</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>SSL VPN 双因子认证（密码+证书）</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>R23</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>基础对象 / 地址对象 / 支持地址组嵌套</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>地址组嵌套 8 层属对象容量</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>R24</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 规则库升级 / 支持通过代理服务器升级规则库</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>F92</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>代理服务器升级规则库属升级方式</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>R25</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 配置锁 / 支持配置锁配置更改锁
+对配置或设备/策略范围加锁，防止并发管理员覆盖</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>F135</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>配置锁（P2 增补功能点）</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>R26</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 带外管理 / 支持基于管理路由发送syslog日志</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>A10+F80</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>带外管理路由 syslog（管理平面策略路由）</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>R27</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 带外管理 / 支持基于管理路由发送管理员认证</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>A10+F80</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>带外管理路由认证</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>R28</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 配置转换 / 支持fortinet配置转换工具</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Fortinet 配置转换工具（配置迁移能力）</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 配置转换 / 支持Palo Alto配置转换工具</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>PA 配置转换工具</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>防火墙管理 / 配置转换 / 支持Hillstone配置转换工具</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>F90</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Hillstone 配置转换工具</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>R31</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>QOS / 拥塞处理 / 支持RED（随机早期检测）</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>B33</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>RED 拥塞处理属 QoS</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>QOS / 拥塞处理 / 支持尾丢弃</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>B33</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>尾丢弃同上</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>R33</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>路由转发 / 组播路由 / 支持IGMP</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>IGMP 属组播路由</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>路由转发 / 组播路由 / 支持MLD</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>MLD（IPv6 组播）</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>R35</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>路由转发 / 组播路由 / 支持PIM-SM</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>PIM-SM</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>R36</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>路由转发 / 组播路由 / 支持PIM-DM</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>A23</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>PIM-DM</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>R37</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>安全控制 / 访问控制 / 访问控制策略支持配置源、目的域名</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>A2+A5</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>策略源/目的域名（地址对象域名支持）</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>R38</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>安全控制 / IPS / 支持基于组播报文作IPS检测</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>C39+A23</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>组播报文 IPS 检测</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>R39</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>安全控制 / DNS / 支持基于域名分类的访问控制</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>域名分类访问控制（URL 分类）</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>R40</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>安全控制 / HTTP3 / 支持基于支持HTTP3的waf功能</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>C53+B28</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>HTTP3/QUIC WAF（QUIC 识别+解密）</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>R41</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>安全控制 / XFF策略 / 支持解析X-Forwarded-For中的原始客户端IP并上报日志</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>C53+F84</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>XFF 原始 IP 解析上报</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>R42</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>安全控制 / 云沙箱 / 支持云沙箱联动功能</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>C46</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>云沙箱联动</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>R43</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>界面 / 英文 / web界面支持英文模式</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>F80</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Web 界面英文模式</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>R44</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>界面 / 英文 / 规则库支持英文</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>B24+F92</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>规则库英文（应用/IPS/AV/IP归属地）</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>R45</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>界面 / 英文 / 可提供英文版用户手册</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>F80</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>英文版用户手册</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>R46</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>界面 / 英文 / 日志支持英文</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>F84</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>日志英文</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>R47</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>界面 / 英文 / 报表支持英文</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>F86</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>报表英文</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>R48</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>硬件加速 / 硬件加速 / 支持网络层加速</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>G95/G97</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>网络层硬件加速（ASIC）——仅能力有无对比，不做性能数值对比</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>R49</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>硬件加速 / 硬件加速 / 支持IPS加速</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>G97</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>IPS 内容加速卡</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>R50</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>硬件加速 / 硬件加速 / 支持DLP content check</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>G97</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>DLP 内容检查加速卡</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>R51</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>硬件加速 / 硬件加速 / 支持ipsec硬件加速</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>G97</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>IPSec 硬件加速卡</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>R52</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>HA / 配置同步 / 配置同步支持整机同步和策略同步</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>F87+F88</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>HA 配置同步（整机/策略）</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>R53</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>HA / 虚系统之间高可用 / 支持在两台物理防火墙之间的虚系统高可用</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>A19+F87</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>虚系统 HA（双活虚系统互备）</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>R54</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>NAT / 策略组 / 每个NAT策略组最大支持512条NAT策略</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>NAT 策略组容量 512 条</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>R55</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>硬件 / 接口支持 / 国产和非国产型号</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>G96</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>25G/40G/2.5G/5G/10G 接口支持</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>R56</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>硬件 / 接口信息 / 硬件支持查看接口光衰信息</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>G96</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>接口光衰信息查看</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>R57</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>ipsec / ipsec / 支持IPSESC链路自動切換</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>E77+A10</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>IPSec 链路自动切换（DPD+策略路由）</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>R58</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>端口镜像 / 端口镜像 / 支持解密端口镜像流量，将解密后的明文流量镜像到专用接口供取证或第三方分析</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>B124</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>解密端口镜像（P2 增补功能点）</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>待P3填充</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete PA vs Topsec firewall comparison deliverables
Add final comparison report assets:
- Add final deliverable Excel with formatted sheets and version header
- Add standalone HTML analysis report with 3 charts and full localization
- Add 8 Python automation scripts for matrix filling, stats, exports, validation
- Add generated dump files for requirements mapping, stats, and report materials
- Add JetBrains Mono font assets for HTML report
- Update comparison documentation with completed P4 phase work

The commit delivers the full P4 phase output for the Hong Kong/Macau PA replacement project, including fully populated functional comparison matrix, requirement mappings, statistical analysis, and polished public-facing report.
</commit_message>
<xml_diff>
--- a/对比工作底稿.xlsx
+++ b/对比工作底稿.xlsx
@@ -285,294 +285,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing_wm1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing_wm6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="6800000" y="6400000"/>
-    <xdr:ext cx="2200000" cy="350000"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Watermark"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm rot="0">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2200000" cy="350000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="b" lIns="0" tIns="0" rIns="0" bIns="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="r"/>
-          <a:r>
-            <a:rPr lang="zh-CN" sz="1600" dirty="0">
-              <a:solidFill>
-                <a:srgbClr val="808080">
-                  <a:alpha val="19999"/>
-                </a:srgbClr>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="SimSun"/>
-            </a:rPr>
-            <a:t>AI 生成</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -857,7 +569,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -991,7 +703,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底交付）</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -999,13 +711,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="4" t="inlineStr"/>
-      <c r="L4" s="4" t="inlineStr"/>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr"/>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同：F84双侧完全支持（TS外发邮件账户+PA邮件通知）；SMTPS加密细节待实测→V清单</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>[R1→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1035,7 +775,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>已支持</t>
+          <t>已支持（原表备注：1、restful api和ansible已按成，可交付；2、firemon已支持，FireMon官网支持列表中，已包含Topsec。实际项目中如遇到有问题，可按项目具体对接、情况调整对接接口）</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -1043,13 +783,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr"/>
-      <c r="N5" s="5" t="inlineStr"/>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>无公开XML/REST API文档（CHM仅"第三方管理接口"概述一句；态势感知联动经SSH superman拉取配置，非标准API）</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>XML API+REST API双通道；API密钥生命周期管理（0-525600分钟）；角色可分别控制Web UI/XML API/CLI/REST API权限；User-ID XML API用户映射集成</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>天融信缺口：F83：TS无公开XML/REST API文档（CHM仅"第三方管理接口"），FireMon对接依赖API通道</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>[R2→主证据矩阵#83] 天融信CHM:功能和特点[toc462736546]第三方管理接口+与态势感知系统联动[-ngfw]；PA:admin p125/p854-858，webhelp p628/p731-732</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1075,13 +843,41 @@
       <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="4" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>无公开XML/REST API文档（CHM仅"第三方管理接口"概述一句；态势感知联动经SSH superman拉取配置，非标准API）</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>XML API+REST API双通道；API密钥生命周期管理（0-525600分钟）；角色可分别控制Web UI/XML API/CLI/REST API权限；User-ID XML API用户映射集成</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>天融信缺口：F83：Ansible经API+Playbook对接同受API缺口影响</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>[R3→主证据矩阵#83] 天融信CHM:功能和特点[toc462736546]第三方管理接口+与态势感知系统联动[-ngfw]；PA:admin p125/p854-858，webhelp p628/p731-732</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1107,13 +903,41 @@
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>无公开XML/REST API文档（CHM仅"第三方管理接口"概述一句；态势感知联动经SSH superman拉取配置，非标准API）</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>XML API+REST API双通道；API密钥生命周期管理（0-525600分钟）；角色可分别控制Web UI/XML API/CLI/REST API权限；User-ID XML API用户映射集成</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>天融信缺口：F83：RESTful API为R2/R3的总通道，PA XML+REST双API完全支持</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>[R4→主证据矩阵#83] 天融信CHM:功能和特点[toc462736546]第三方管理接口+与态势感知系统联动[-ngfw]；PA:admin p125/p854-858，webhelp p628/p731-732</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1143,7 +967,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底交付）</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1151,13 +975,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
-      <c r="L8" s="4" t="inlineStr"/>
-      <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" s="4" t="inlineStr"/>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同：F84：TS日志查看+PA日志筛选均支持；源/目的IP字段级过滤待实测→V清单</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>[R5→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1183,13 +1035,41 @@
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr"/>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同：同R5（目的IP过滤）</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>[R6→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1215,13 +1095,41 @@
       <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr"/>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同：同R5（源端口过滤）</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>[R7→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1247,13 +1155,41 @@
       <c r="E11" s="5" t="inlineStr"/>
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="inlineStr"/>
-      <c r="L11" s="5" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr"/>
-      <c r="N11" s="5" t="inlineStr"/>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同：同R5（目的端口过滤）</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>[R8→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1275,13 +1211,41 @@
       <c r="E12" s="4" t="inlineStr"/>
       <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：F84：PA日志字段体系有据（会话开始/结束时间）；TS连接日志字段明细待实测→V清单</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>[R9→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1303,13 +1267,41 @@
       <c r="E13" s="5" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr"/>
-      <c r="L13" s="5" t="inlineStr"/>
-      <c r="M13" s="5" t="inlineStr"/>
-      <c r="N13" s="5" t="inlineStr"/>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：同R9（会话结束时间）</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>[R10→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1331,13 +1323,41 @@
       <c r="E14" s="4" t="inlineStr"/>
       <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
-      <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="inlineStr"/>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：同R9：PA解密日志含结束原因字段；TS待实测</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>[R11→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1367,7 +1387,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>已交付</t>
+          <t>已交付（原表备注：产线已提供可平滑升级的模块和规则库给前方）</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1375,13 +1395,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
-      <c r="K15" s="5" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr"/>
-      <c r="M15" s="5" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr"/>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>License许可证文件模式：受限制模块授权（升级中心&gt;License升级）；功能模块化授权；到期后行为未见说明</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>需订阅授权</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>订阅制：授权码激活订阅（威胁防护/DNS安全/WildFire/UEBA/SaaS安全等）；到期前30天告警；到期后订阅功能停止执行、基础防火墙继续运行；解密镜像免费许可证机制</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>实现路径不同：F91：TS License升级+PA订阅续期；升级不中断业务待实测→V清单</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>[R12→主证据矩阵#91] 天融信CHM:选项[topic206]License升级；PA:webhelp p851，admin p76-78</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1411,7 +1459,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>部分交付</t>
+          <t>部分交付（原表备注：当前规则库已支持：Facebook、YouTube、Twitter、WhatsApp、office365（库中协议名：微软通用服务）、Tiktok、Zoom、Steam、TeamView协议、Telegram；20260710：；前方反馈增加应用：Threads、Instagram、Linkedln、Snapchat、LINE、Microsoft Teams、Twitch、EPIC、Google Gemini、Open Chat；20260717：；snapchat、Twitch、EPIC计划7月底发布的规则库会支持；OpenChat暂不支持，需要抓包分析；其余协议已支持）</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1419,13 +1467,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：PA App-ID全球库；TS国际应用（Facebook）识别覆盖待抽样实测→V清单</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>[R13→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1447,13 +1523,41 @@
       <c r="E17" s="5" t="inlineStr"/>
       <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr"/>
-      <c r="K17" s="5" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr"/>
-      <c r="M17" s="5" t="inlineStr"/>
-      <c r="N17" s="5" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：YouTube，同R13港澳应用抽样清单</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>[R14→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1475,13 +1579,41 @@
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：Twitter(X)，同R13</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>[R15→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1503,13 +1635,41 @@
       <c r="E19" s="5" t="inlineStr"/>
       <c r="F19" s="5" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr"/>
-      <c r="K19" s="5" t="inlineStr"/>
-      <c r="L19" s="5" t="inlineStr"/>
-      <c r="M19" s="5" t="inlineStr"/>
-      <c r="N19" s="5" t="inlineStr"/>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：WhatsApp，同R13</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>[R16→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1531,13 +1691,41 @@
       <c r="E20" s="4" t="inlineStr"/>
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：TikTok，同R13</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>[R17→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1559,13 +1747,41 @@
       <c r="E21" s="5" t="inlineStr"/>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr"/>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr"/>
-      <c r="K21" s="5" t="inlineStr"/>
-      <c r="L21" s="5" t="inlineStr"/>
-      <c r="M21" s="5" t="inlineStr"/>
-      <c r="N21" s="5" t="inlineStr"/>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：Zoom，同R13</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>[R18→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1587,13 +1803,41 @@
       <c r="E22" s="4" t="inlineStr"/>
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="4" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="4" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="4" t="inlineStr"/>
-      <c r="L22" s="4" t="inlineStr"/>
-      <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr"/>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：Steam，同R13</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>[R19→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1615,13 +1859,41 @@
       <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr"/>
-      <c r="K23" s="5" t="inlineStr"/>
-      <c r="L23" s="5" t="inlineStr"/>
-      <c r="M23" s="5" t="inlineStr"/>
-      <c r="N23" s="5" t="inlineStr"/>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B27+B36：Office365含子应用识别；TS覆盖待实测</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>[R20→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1643,13 +1915,41 @@
       <c r="E24" s="4" t="inlineStr"/>
       <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="4" t="inlineStr"/>
-      <c r="L24" s="4" t="inlineStr"/>
-      <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr"/>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：B24+B36：TeamViewer，同R13</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>[R21→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1679,7 +1979,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：已提交需求，待接入产线确认合入时间点）</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1687,13 +1987,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr"/>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="5" t="inlineStr"/>
-      <c r="K25" s="5" t="inlineStr"/>
-      <c r="L25" s="5" t="inlineStr"/>
-      <c r="M25" s="5" t="inlineStr"/>
-      <c r="N25" s="5" t="inlineStr"/>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>单因子（密码/证书）+双因子（密码+证书/密码+UKey/密码+短信）；短信网关配置；UKey USB认证（需驱动）</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>MFA 供应商API集成（Okta/RSA SecurID/PingID等，随内容更新扩充）；RADIUS/SAML/Kerberos；GlobalProtect网关入站MFA提示</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>PA优势：E74：TS密码+证书/UKey/短信与PA MFA供应商体系均完全支持</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>[R22→主证据矩阵#74] 天融信CHM:账号管理[topic53]+Local服务器[toc462834527]+短信[topic68]；PA:webhelp p839/p741/admin p236-240</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1723,7 +2051,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1731,13 +2059,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>访问控制策略数量受 license 控制[toc450050600]；具体容量数值官方文档未公开</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>策略/对象容量因型号而异（见各型号 Datasheet）；地址组嵌套等容量项在 datasheet 规格表</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：A5：地址组嵌套层数（8层）属容量规格，双方需查datasheet→V清单</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>[R23→主证据矩阵#5] 天融信CHM:配置访问控制策略；PA:Datasheet 规格表</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1767,7 +2123,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -1775,13 +2131,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr"/>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr"/>
-      <c r="K27" s="5" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr"/>
-      <c r="M27" s="5" t="inlineStr"/>
-      <c r="N27" s="5" t="inlineStr"/>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>升级中心四件套：固件维护（当前固件/Patch列表/固件升级/版本说明）+引擎管理（引擎模块单独升级/新模块安装免整机升级）+规则库升级（应用识别/IPS/URL/APT/僵木蠕/病毒）+License升级</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Device&gt;Software（检查更新/下载/上传/安装/删除映像，发行说明）；动态内容更新（防病毒/应用程序/威胁内容版本）；Panorama统一软件更新管理（验证+分批）</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：F92：TS升级服务器+PA更新服务器均支持；经代理服务器升级双方手册未载→V清单</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>[R24→主证据矩阵#92] 天融信CHM:固件维护[topic83]+引擎管理[topic84]+规则库升级[toc462834565]；PA:webhelp p846-847/p1091，admin p33</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1804,13 +2188,41 @@
       <c r="E28" s="4" t="inlineStr"/>
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr"/>
-      <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>不支持</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>无配置锁/并发编辑控制机制（检索无命中，否定证据；仅登录失败锁定等账户策略）</t>
+        </is>
+      </c>
+      <c r="J28" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>配置更改限制锁：Config Lock（阻止他人更改待选配置）+Commit Lock（阻止提交）两种类型；锁定备注+锁定图标与计数；多管理员部分保存/提交范围控制</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>天融信缺口：F135：TS无配置锁机制（检索无命中）；PA Config Lock/Commit Lock完全支持——PA优势</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>[R25→主证据矩阵#135] 天融信CHM:登录安全策略[ref465087238]（仅账户级）；PA:webhelp p40，admin p100-101</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1840,7 +2252,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -1848,13 +2260,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr"/>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="5" t="inlineStr"/>
-      <c r="K29" s="5" t="inlineStr"/>
-      <c r="L29" s="5" t="inlineStr"/>
-      <c r="M29" s="5" t="inlineStr"/>
-      <c r="N29" s="5" t="inlineStr"/>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>策略路由：按源/目的地址端口、ISP名称、协议、角色等选路；路由优先级：回环&gt;黑洞&gt;直连&gt;策略路由&gt;ISP路由&gt;静态&gt;动态</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>PBF 基于策略的转发：源区域/地址/用户/应用/服务+下一跳；支持路径监控与失效切换；BFD</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>实现路径不同：A10+F80：TS独立管理路由分离显式支持；PA MGT带外+服务路由</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>[R26→主证据矩阵#10] 天融信CHM:策略路由[toc490041605]+路由[ref487714854]；PA:webhelp p156 PBF</t>
+        </is>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1876,13 +2316,41 @@
       <c r="E30" s="4" t="inlineStr"/>
       <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="4" t="inlineStr"/>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="4" t="inlineStr"/>
-      <c r="L30" s="4" t="inlineStr"/>
-      <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr"/>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>策略路由：按源/目的地址端口、ISP名称、协议、角色等选路；路由优先级：回环&gt;黑洞&gt;直连&gt;策略路由&gt;ISP路由&gt;静态&gt;动态</t>
+        </is>
+      </c>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>PBF 基于策略的转发：源区域/地址/用户/应用/服务+下一跳；支持路径监控与失效切换；BFD</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>实现路径不同：A10+F80：带外管理认证路由同R26</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>[R27→主证据矩阵#10] 天融信CHM:策略路由[toc490041605]+路由[ref487714854]；PA:webhelp p156 PBF</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1913,7 +2381,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>已交付</t>
+          <t>已交付（原表备注：2026年8月底）</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -1921,13 +2389,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr"/>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr"/>
-      <c r="M31" s="5" t="inlineStr"/>
-      <c r="N31" s="5" t="inlineStr"/>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>配置文件导入导出（导入可设为启动配置）；用户批量导入（TXT/CSV模板）；证书导入导出（PKCS12/加密密码）；日志导出CSV/TXT</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>导出设备状态/设备配置包（FW主密钥加密）；导出命名配置快照（XML）；导入设备状态（迁移/更换设备）；阻止私钥导出选项</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：F90：双方手册均无第三方配置转换工具章节；需查迁移工具（PA Expedition/天融信迁移工具）→V清单</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>[R28→主证据矩阵#90] 天融信CHM:配置维护[toc462834560]+管理用户[ref467487317]+CA管理[ca3]；PA:webhelp p653，admin p106-107/p1049</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1965,13 +2461,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr"/>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="4" t="inlineStr"/>
-      <c r="L32" s="4" t="inlineStr"/>
-      <c r="M32" s="4" t="inlineStr"/>
-      <c r="N32" s="4" t="inlineStr"/>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>配置文件导入导出（导入可设为启动配置）；用户批量导入（TXT/CSV模板）；证书导入导出（PKCS12/加密密码）；日志导出CSV/TXT</t>
+        </is>
+      </c>
+      <c r="J32" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>导出设备状态/设备配置包（FW主密钥加密）；导出命名配置快照（XML）；导入设备状态（迁移/更换设备）；阻止私钥导出选项</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：F90：PA配置转换（本替代项目反向场景：PA→天融信工具为关键）→V清单</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>[R29→主证据矩阵#90] 天融信CHM:配置维护[toc462834560]+管理用户[ref467487317]+CA管理[ca3]；PA:webhelp p653，admin p106-107/p1049</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2009,13 +2533,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr"/>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr"/>
-      <c r="K33" s="5" t="inlineStr"/>
-      <c r="L33" s="5" t="inlineStr"/>
-      <c r="M33" s="5" t="inlineStr"/>
-      <c r="N33" s="5" t="inlineStr"/>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>配置文件导入导出（导入可设为启动配置）；用户批量导入（TXT/CSV模板）；证书导入导出（PKCS12/加密密码）；日志导出CSV/TXT</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>导出设备状态/设备配置包（FW主密钥加密）；导出命名配置快照（XML）；导入设备状态（迁移/更换设备）；阻止私钥导出选项</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：F90：Hillstone转换工具同R28</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>[R30→主证据矩阵#90] 天融信CHM:配置维护[toc462834560]+管理用户[ref467487317]+CA管理[ca3]；PA:webhelp p653，admin p106-107/p1049</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2045,7 +2597,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底（常规化））</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2053,13 +2605,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr"/>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="4" t="inlineStr"/>
-      <c r="L34" s="4" t="inlineStr"/>
-      <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr"/>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>虚拟通道：保证带宽（最低可用带宽）+最大带宽限制；虚拟链路上/下行总带宽策略</t>
+        </is>
+      </c>
+      <c r="J34" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>QoS 配置文件：每类 Egress Guaranteed（保障速率%）+Egress Max（最大速率）+突发</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：B33：双方QoS完全支持；RED/尾丢弃队列算法细节未载→V清单</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>[R31→主证据矩阵#33] 天融信CHM:配置流量策略[toc399440500]；PA:webhelp p609/admin p1125</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2081,13 +2661,41 @@
       <c r="E35" s="5" t="inlineStr"/>
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="5" t="inlineStr"/>
-      <c r="H35" s="5" t="inlineStr"/>
-      <c r="I35" s="5" t="inlineStr"/>
-      <c r="J35" s="5" t="inlineStr"/>
-      <c r="K35" s="5" t="inlineStr"/>
-      <c r="L35" s="5" t="inlineStr"/>
-      <c r="M35" s="5" t="inlineStr"/>
-      <c r="N35" s="5" t="inlineStr"/>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>虚拟通道：保证带宽（最低可用带宽）+最大带宽限制；虚拟链路上/下行总带宽策略</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>QoS 配置文件：每类 Egress Guaranteed（保障速率%）+Egress Max（最大速率）+突发</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：B33：尾丢弃同R31</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>[R32→主证据矩阵#33] 天融信CHM:配置流量策略[toc399440500]；PA:webhelp p609/admin p1125</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2113,7 +2721,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2121,13 +2729,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr"/>
-      <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="4" t="inlineStr"/>
-      <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr"/>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>IPv4组播(PIM)+IPv6组播；组播转发表项；组播报文IPS检测（R38需求）</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>IP多播：PIM-SM(ASM)/SSM+IGMP+静态RP/BSR/自动RP；MSDP；PIM-DM 未见——待验证</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>天融信优势：A23：TS组播路由完全支持/PA部分支持；IGMP随A23证据</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>[R33→主证据矩阵#23] 天融信CHM:IPv4组播[ipv4.html]；PA:webhelp p469-472 多播</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -2149,13 +2785,41 @@
       <c r="E37" s="5" t="inlineStr"/>
       <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr"/>
-      <c r="H37" s="5" t="inlineStr"/>
-      <c r="I37" s="5" t="inlineStr"/>
-      <c r="J37" s="5" t="inlineStr"/>
-      <c r="K37" s="5" t="inlineStr"/>
-      <c r="L37" s="5" t="inlineStr"/>
-      <c r="M37" s="5" t="inlineStr"/>
-      <c r="N37" s="5" t="inlineStr"/>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>IPv4组播(PIM)+IPv6组播；组播转发表项；组播报文IPS检测（R38需求）</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>IP多播：PIM-SM(ASM)/SSM+IGMP+静态RP/BSR/自动RP；MSDP；PIM-DM 未见——待验证</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>天融信优势：A23：MLD（IPv6组播）随A23</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>[R34→主证据矩阵#23] 天融信CHM:IPv4组播[ipv4.html]；PA:webhelp p469-472 多播</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2177,13 +2841,41 @@
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr"/>
       <c r="G38" s="4" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr"/>
-      <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="4" t="inlineStr"/>
-      <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr"/>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>IPv4组播(PIM)+IPv6组播；组播转发表项；组播报文IPS检测（R38需求）</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>IP多播：PIM-SM(ASM)/SSM+IGMP+静态RP/BSR/自动RP；MSDP；PIM-DM 未见——待验证</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>天融信优势：A23：PIM-SM随A23</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>[R35→主证据矩阵#23] 天融信CHM:IPv4组播[ipv4.html]；PA:webhelp p469-472 多播</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2205,13 +2897,41 @@
       <c r="E39" s="5" t="inlineStr"/>
       <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr"/>
-      <c r="H39" s="5" t="inlineStr"/>
-      <c r="I39" s="5" t="inlineStr"/>
-      <c r="J39" s="5" t="inlineStr"/>
-      <c r="K39" s="5" t="inlineStr"/>
-      <c r="L39" s="5" t="inlineStr"/>
-      <c r="M39" s="5" t="inlineStr"/>
-      <c r="N39" s="5" t="inlineStr"/>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>IPv4组播(PIM)+IPv6组播；组播转发表项；组播报文IPS检测（R38需求）</t>
+        </is>
+      </c>
+      <c r="J39" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>IP多播：PIM-SM(ASM)/SSM+IGMP+静态RP/BSR/自动RP；MSDP；PIM-DM 未见——待验证</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>天融信优势：A23：PIM-DM随A23</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>[R36→主证据矩阵#23] 天融信CHM:IPv4组播[ipv4.html]；PA:webhelp p469-472 多播</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2237,7 +2957,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2245,13 +2965,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr"/>
-      <c r="J40" s="4" t="inlineStr"/>
-      <c r="K40" s="4" t="inlineStr"/>
-      <c r="L40" s="4" t="inlineStr"/>
-      <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" s="4" t="inlineStr"/>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改+自定义应用+应用组；应用作为策略过滤条件</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>App-ID 识别引擎（应用+容器+依赖应用+子应用分级）；应用程序过滤器/组；ACE 云引擎未知应用检测</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>实现路径不同：A2+A5：策略源/目的域名（TS域名对象+PA FQDN对象）</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>[R37→主证据矩阵#2] 天融信CHM:应用[toc448912175]+预定义应用[topic194]；PA:admin p920-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2277,13 +3025,41 @@
       </c>
       <c r="F41" s="5" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr"/>
-      <c r="H41" s="5" t="inlineStr"/>
-      <c r="I41" s="5" t="inlineStr"/>
-      <c r="J41" s="5" t="inlineStr"/>
-      <c r="K41" s="5" t="inlineStr"/>
-      <c r="L41" s="5" t="inlineStr"/>
-      <c r="M41" s="5" t="inlineStr"/>
-      <c r="N41" s="5" t="inlineStr"/>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>入侵防御模块内置规则集（预定义+自定义规则+白名单），规则库经升级中心在线/离线更新；特征条数官方文档未公布，P3 从产品彩页/规格页核实</t>
+        </is>
+      </c>
+      <c r="J41" s="16" t="inlineStr">
+        <is>
+          <t>需订阅授权</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>Threat Prevention 订阅；Vulnerability Protection（防漏洞）+Anti-Spyware（防间谍软件）两配置文件；特征库经 Dynamic Updates 更新</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>天融信优势（待实测）：C39+A23：组播报文IPS检测双方手册未显式载明→V清单</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>[R38→主证据矩阵#39] 天融信CHM:入侵防御[topic10/200-202]+升级中心[topic61]；PA:Web帮助&gt;安全配置文件&gt;Vulnerability/Anti-Spyware+Device&gt;Dynamic Updates</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2313,7 +3089,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>已交付</t>
+          <t>已交付（原表备注：已交付）</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2321,13 +3097,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="inlineStr"/>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="4" t="inlineStr"/>
-      <c r="M42" s="4" t="inlineStr"/>
-      <c r="N42" s="4" t="inlineStr"/>
+      <c r="H42" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>URL分类库：系统内置+自定义URL组；预定义分类页签+全局查询；分类数/库规模未在手册公布——待实测</t>
+        </is>
+      </c>
+      <c r="J42" s="16" t="inlineStr">
+        <is>
+          <t>需订阅授权</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>PAN-DB 订阅数据库（URL 过滤已并入高级URL过滤订阅）；预定义类别列表+URL/IP云数据库；PAN-DB 私有云选项</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>实现路径不同：D57：TS内置分类库/PA PAN-DB订阅，实现路径不同</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>[R39→主证据矩阵#57] 天融信CHM:URL分类[toc448912180]+预定义分类[topic191]；PA:webhelp p273-275/admin p73</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -2357,7 +3161,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>待评估（原表备注：已提交需求，等待WAF答复）</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
@@ -2365,13 +3169,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr"/>
-      <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="5" t="inlineStr"/>
-      <c r="K43" s="5" t="inlineStr"/>
-      <c r="L43" s="5" t="inlineStr"/>
-      <c r="M43" s="5" t="inlineStr"/>
-      <c r="N43" s="5" t="inlineStr"/>
+      <c r="H43" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>WAF 模块：预定义核心规则库（多语言通用+CMS专项 phpwind/wordpress/discuz）+自定义规则；爬虫管理（内置爬虫库+自定义）；登录页面防护（basic/get/form/digest 暴力登录拦截）；IP黑白名单；SSL解密代理WAF；与TopWAF联动</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>无独立 WAF 模块；Web 攻击防护经漏洞保护签名（SQL注入/命令注入）+内联云分析（深度学习实时检测 SQL/命令注入）；XSS/爬虫/登录防护专项未见；钓鱼防护依赖高级URL过滤</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>天融信优势（待实测）：C53+B28：PA手册建议阻止QUIC（无法解密）；HTTP3解密WAF双方均未见→V清单</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>[R40→主证据矩阵#53] 天融信CHM:WAF[anquancelue_waf]+爬虫[topic220]+登录页面[topic222]；PA:webhelp p270（否定证据：中文手册无WAF专章）</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2393,13 +3225,41 @@
       <c r="E44" s="4" t="inlineStr"/>
       <c r="F44" s="4" t="inlineStr"/>
       <c r="G44" s="4" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr"/>
-      <c r="J44" s="4" t="inlineStr"/>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="4" t="inlineStr"/>
-      <c r="M44" s="4" t="inlineStr"/>
-      <c r="N44" s="4" t="inlineStr"/>
+      <c r="H44" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>WAF 模块：预定义核心规则库（多语言通用+CMS专项 phpwind/wordpress/discuz）+自定义规则；爬虫管理（内置爬虫库+自定义）；登录页面防护（basic/get/form/digest 暴力登录拦截）；IP黑白名单；SSL解密代理WAF；与TopWAF联动</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>无独立 WAF 模块；Web 攻击防护经漏洞保护签名（SQL注入/命令注入）+内联云分析（深度学习实时检测 SQL/命令注入）；XSS/爬虫/登录防护专项未见；钓鱼防护依赖高级URL过滤</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>天融信优势（待实测）：C53+F84：XFF原始IP解析上报双方手册未载→V清单</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>[R41→主证据矩阵#53] 天融信CHM:WAF[anquancelue_waf]+爬虫[topic220]+登录页面[topic222]；PA:webhelp p270（否定证据：中文手册无WAF专章）</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -2425,7 +3285,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>不支持</t>
+          <t>不支持（原表备注：公司无云沙箱产品，暂无法支持）</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
@@ -2433,13 +3293,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
-      <c r="J45" s="5" t="inlineStr"/>
-      <c r="K45" s="5" t="inlineStr"/>
-      <c r="L45" s="5" t="inlineStr"/>
-      <c r="M45" s="5" t="inlineStr"/>
-      <c r="N45" s="5" t="inlineStr"/>
+      <c r="H45" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>APT联动配置：按工作模式（深度/智能模式）决定是否送沙箱；沙箱返回 MD5+判定结果，恶意文件 MD5 记入本地特征库；MD5值查询界面；云安全中心云检测</t>
+        </is>
+      </c>
+      <c r="J45" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>WildFire 分析配置文件：按文件类型/应用/传输方向转发公共云或私有云；免费转发 PE 分析；判定恶意/灰色/良性/钓鱼；新恶意软件生成签名实时分发</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同：C46：TS联动第三方沙箱/PA WildFire云订阅（需订阅授权），仅命名不同</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>[R42→主证据矩阵#46] 天融信CHM:APT联动[apt]+MD5查询[md5]+云安全中心[topic52]；PA:webhelp p283/admin p67-68</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2469,7 +3357,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>已交付</t>
+          <t>已交付（原表备注：2026年4月底（已交付））</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -2477,13 +3365,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="4" t="inlineStr"/>
-      <c r="M46" s="4" t="inlineStr"/>
-      <c r="N46" s="4" t="inlineStr"/>
+      <c r="H46" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Web界面：浏览器HTTPS登录（feth0默认192.168.1.x）；自动保存/系统切换/本地告警/CLI入口等界面功能</t>
+        </is>
+      </c>
+      <c r="J46" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>Web界面：全局查找（跨配置搜索对象/策略/威胁ID）；多语言切换；Panorama与防火墙界面同构</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同（待实测）：F80：PA多语言显式支持；TS界面英文切换待实测→V清单</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>[R43→主证据矩阵#80] 天融信CHM:登录系统[ngfw2]+通过浏览器登录[topic142]+熟悉WEB管理界面[toc490041566]；PA:webhelp p21/p26/p42，admin p89</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2509,7 +3425,7 @@
       <c r="E47" s="5" t="inlineStr"/>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -2517,13 +3433,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr"/>
-      <c r="I47" s="5" t="inlineStr"/>
-      <c r="J47" s="5" t="inlineStr"/>
-      <c r="K47" s="5" t="inlineStr"/>
-      <c r="L47" s="5" t="inlineStr"/>
-      <c r="M47" s="5" t="inlineStr"/>
-      <c r="N47" s="5" t="inlineStr"/>
+      <c r="H47" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>应用类型24大类（父类/子类）；预定义应用不可改；应用识别/IPS/URL/APT/僵木蠕/病毒引擎规则库频繁更新；应用总数官方文档未公布</t>
+        </is>
+      </c>
+      <c r="J47" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>App-ID 每周内容更新；应用程序+过滤器+组三级；ACE 云引擎经 ML 为未知应用生成新 App-ID；具体数量未在手册公布</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>待验证（待实测）：B24+F92：TS日志语言中英文可选；规则库/界面语言待实测</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>[R44→主证据矩阵#24] 天融信CHM:应用[toc448912175]；PA:admin p889-940 App-ID</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -2545,13 +3489,41 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="4" t="inlineStr"/>
       <c r="G48" s="4" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr"/>
-      <c r="J48" s="4" t="inlineStr"/>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="4" t="inlineStr"/>
-      <c r="M48" s="4" t="inlineStr"/>
-      <c r="N48" s="4" t="inlineStr"/>
+      <c r="H48" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Web界面：浏览器HTTPS登录（feth0默认192.168.1.x）；自动保存/系统切换/本地告警/CLI入口等界面功能</t>
+        </is>
+      </c>
+      <c r="J48" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>Web界面：全局查找（跨配置搜索对象/策略/威胁ID）；多语言切换；Panorama与防火墙界面同构</t>
+        </is>
+      </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：F80：PA中英文手册齐备；TS英文版手册需向原厂查询→V清单</t>
+        </is>
+      </c>
+      <c r="M48" s="4" t="inlineStr">
+        <is>
+          <t>[R45→主证据矩阵#80] 天融信CHM:登录系统[ngfw2]+通过浏览器登录[topic142]+熟悉WEB管理界面[toc490041566]；PA:webhelp p21/p26/p42，admin p89</t>
+        </is>
+      </c>
+      <c r="N48" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -2573,7 +3545,7 @@
       <c r="E49" s="5" t="inlineStr"/>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
@@ -2581,13 +3553,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr"/>
-      <c r="I49" s="5" t="inlineStr"/>
-      <c r="J49" s="5" t="inlineStr"/>
-      <c r="K49" s="5" t="inlineStr"/>
-      <c r="L49" s="5" t="inlineStr"/>
-      <c r="M49" s="5" t="inlineStr"/>
-      <c r="N49" s="5" t="inlineStr"/>
+      <c r="H49" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>日志配置（本地存储与外发级别分别设置）；日志服务器syslog外发；日志存储管理（容量上限/每日每周备份/FTP备份/按天导出/加密GB2312-UTF8）</t>
+        </is>
+      </c>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>日志设置+日志转发配置文件（挂安全/DoS/隧道策略）；转发目标：Panorama/日志记录服务/syslog/SNMP陷阱/邮件/HTTP(S)；LFC日志转发卡（硬件加速）</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>仅命名不同：F84：TS日志语言中/英文可选显式支持；PA英文原生</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>[R46→主证据矩阵#84] 天融信CHM:日志配置[toc490041759]+日志服务器配置[ref465084227]+日志存储管理[topic212]；PA:webhelp p305/p808/p817/p721，admin p579/p589</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -2609,7 +3609,7 @@
       <c r="E50" s="4" t="inlineStr"/>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
@@ -2617,13 +3617,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="4" t="inlineStr"/>
-      <c r="J50" s="4" t="inlineStr"/>
-      <c r="K50" s="4" t="inlineStr"/>
-      <c r="L50" s="4" t="inlineStr"/>
-      <c r="M50" s="4" t="inlineStr"/>
-      <c r="N50" s="4" t="inlineStr"/>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>报表模块：报表配置+报表模板自定义（模板管理页签）；威胁统计多视图；攻击者/受害者关联分析（攻击链支持）+数据导出</t>
+        </is>
+      </c>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>40+预定义报告+自定义报告（按需/每夜计划运行）；报告组聚合PDF（含标题页）+计划邮件投递；报告存储约200MB配额管理</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>实现路径不同（待实测）：F86：报表英文输出TS待实测</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>[R47→主证据矩阵#86] 天融信CHM:报表配置[topic21]+模板管理[topic23]+攻击者[topic55]；PA:webhelp p107/p109，admin p553-570</t>
+        </is>
+      </c>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -2658,13 +3686,41 @@
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
-      <c r="H51" s="5" t="inlineStr"/>
-      <c r="I51" s="5" t="inlineStr"/>
-      <c r="J51" s="5" t="inlineStr"/>
-      <c r="K51" s="5" t="inlineStr"/>
-      <c r="L51" s="5" t="inlineStr"/>
-      <c r="M51" s="5" t="inlineStr"/>
-      <c r="N51" s="5" t="inlineStr"/>
+      <c r="H51" s="14" t="inlineStr">
+        <is>
+          <t>待验证</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>CHM不列型号梯度（系统组成仅描述1U/2U形态与3.2294软件平台）；天融信NGFW全系列型号与规格需查产品手册</t>
+        </is>
+      </c>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>手册全篇引用型号体系：PA-220/400/800/3200/3400/5200/5400/7000系列+PA-7500+CN系列（容器防火墙集群）+VM系列；型号间能力差异显式标注（BFD最小间隔/vsys基数/HA3聚合等）</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：G97：网络层/IPS/DLP/IPSec加速能力属硬件规格，需查双方datasheet→V清单</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>[R48→主证据矩阵#95] 天融信CHM:系统组成[topic32]（型号信息缺失）；PA:webhelp p526/p1018，admin p379/p1312</t>
+        </is>
+      </c>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -2698,13 +3754,41 @@
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
-      <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="4" t="inlineStr"/>
-      <c r="J52" s="4" t="inlineStr"/>
-      <c r="K52" s="4" t="inlineStr"/>
-      <c r="L52" s="4" t="inlineStr"/>
-      <c r="M52" s="4" t="inlineStr"/>
-      <c r="N52" s="4" t="inlineStr"/>
+      <c r="H52" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>系统组成：扩展插槽用于扩展卡安装（不同NGFW产品支持不同数量的扩展模块）</t>
+        </is>
+      </c>
+      <c r="J52" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>PA-7000系列模块化机箱（NPC/LPC插槽，日志卡LFC槽位）；中低端型号为一体化固定接口，扩展性需查硬件参考指南</t>
+        </is>
+      </c>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：G97：IPS加速同R48</t>
+        </is>
+      </c>
+      <c r="M52" s="4" t="inlineStr">
+        <is>
+          <t>[R49→主证据矩阵#97] 天融信CHM:系统组成[topic32]；PA:admin p329/p477/p1329（插槽表述仅限PA-7000）</t>
+        </is>
+      </c>
+      <c r="N52" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -2738,13 +3822,41 @@
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
-      <c r="H53" s="5" t="inlineStr"/>
-      <c r="I53" s="5" t="inlineStr"/>
-      <c r="J53" s="5" t="inlineStr"/>
-      <c r="K53" s="5" t="inlineStr"/>
-      <c r="L53" s="5" t="inlineStr"/>
-      <c r="M53" s="5" t="inlineStr"/>
-      <c r="N53" s="5" t="inlineStr"/>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>系统组成：扩展插槽用于扩展卡安装（不同NGFW产品支持不同数量的扩展模块）</t>
+        </is>
+      </c>
+      <c r="J53" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>PA-7000系列模块化机箱（NPC/LPC插槽，日志卡LFC槽位）；中低端型号为一体化固定接口，扩展性需查硬件参考指南</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：G97：DLP内容检查加速同R48</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>[R50→主证据矩阵#97] 天融信CHM:系统组成[topic32]；PA:admin p329/p477/p1329（插槽表述仅限PA-7000）</t>
+        </is>
+      </c>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -2775,7 +3887,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2027年2月交付）</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -2783,13 +3895,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="4" t="inlineStr"/>
-      <c r="J54" s="4" t="inlineStr"/>
-      <c r="K54" s="4" t="inlineStr"/>
-      <c r="L54" s="4" t="inlineStr"/>
-      <c r="M54" s="4" t="inlineStr"/>
-      <c r="N54" s="4" t="inlineStr"/>
+      <c r="H54" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>系统组成：扩展插槽用于扩展卡安装（不同NGFW产品支持不同数量的扩展模块）</t>
+        </is>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>PA-7000系列模块化机箱（NPC/LPC插槽，日志卡LFC槽位）；中低端型号为一体化固定接口，扩展性需查硬件参考指南</t>
+        </is>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：G97：IPSec硬件加速同R48</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>[R51→主证据矩阵#97] 天融信CHM:系统组成[topic32]；PA:admin p329/p477/p1329（插槽表述仅限PA-7000）</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -2815,7 +3955,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>待交付</t>
+          <t>待交付（原表备注：2026年9月底）</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
@@ -2823,13 +3963,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr"/>
-      <c r="I55" s="5" t="inlineStr"/>
-      <c r="J55" s="5" t="inlineStr"/>
-      <c r="K55" s="5" t="inlineStr"/>
-      <c r="L55" s="5" t="inlineStr"/>
-      <c r="M55" s="5" t="inlineStr"/>
-      <c r="N55" s="5" t="inlineStr"/>
+      <c r="H55" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>HA四模式：主备（AS）/连接保护/负载均衡/集群模式；心跳口（本端/对端IP）+虚拟ID+监控角色主/备</t>
+        </is>
+      </c>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>主动/被动（A/P）+主动/主动（A/A，会话所有者机制）；HA1控制链路+HA2数据链路（备份链路可选）；HA1加密；专用HA端口（按型号）</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>实现路径不同：F87+F88：TS显式支持整机/策略/管理员/实时四级配置同步；PA配置同步完整</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>[R52→主证据矩阵#87] 天融信CHM:高可用性[toc462834583]+配置[topic15/136/140/141]；PA:admin p377-399/p411，webhelp p706-717</t>
+        </is>
+      </c>
+      <c r="N55" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -2859,7 +4027,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>待评估（原表备注：已提交研究院，等待研究院答复）</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -2867,13 +4035,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="4" t="inlineStr"/>
-      <c r="J56" s="4" t="inlineStr"/>
-      <c r="K56" s="4" t="inlineStr"/>
-      <c r="L56" s="4" t="inlineStr"/>
-      <c r="M56" s="4" t="inlineStr"/>
-      <c r="N56" s="4" t="inlineStr"/>
+      <c r="H56" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>虚系统：路由/非路由模式；虚接口+虚拟链路互联；虚系统管理员（无授权能力）；对象共享/独享</t>
+        </is>
+      </c>
+      <c r="J56" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>vsys：独立策略/接口/管理员；vsys间User-ID数据共享；外部区域/共享网关；高型号需vsyss许可证</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>实现路径不同（待实测）：A19+F87：虚系统级HA（跨设备虚系统互备）双方手册未载→V清单</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>[R53→主证据矩阵#19] 天融信CHM:虚拟系统[xunixitong/topic128]；PA:webhelp p780-781/admin p1312</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -2907,13 +4103,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H57" s="5" t="inlineStr"/>
-      <c r="I57" s="5" t="inlineStr"/>
-      <c r="J57" s="5" t="inlineStr"/>
-      <c r="K57" s="5" t="inlineStr"/>
-      <c r="L57" s="5" t="inlineStr"/>
-      <c r="M57" s="5" t="inlineStr"/>
-      <c r="N57" s="5" t="inlineStr"/>
+      <c r="H57" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>访问控制策略数量受 license 控制[toc450050600]；具体容量数值官方文档未公开</t>
+        </is>
+      </c>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>策略/对象容量因型号而异（见各型号 Datasheet）；地址组嵌套等容量项在 datasheet 规格表</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：A5：NAT策略组容量512条属规格项，需查datasheet</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>[R54→主证据矩阵#5] 天融信CHM:配置访问控制策略；PA:Datasheet 规格表</t>
+        </is>
+      </c>
+      <c r="N57" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -2943,19 +4167,51 @@
           <t>高</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>（原表备注：待有项目后反馈产线评估）</t>
+        </is>
+      </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
           <t>产品线</t>
         </is>
       </c>
-      <c r="H58" s="4" t="inlineStr"/>
-      <c r="I58" s="4" t="inlineStr"/>
-      <c r="J58" s="4" t="inlineStr"/>
-      <c r="K58" s="4" t="inlineStr"/>
-      <c r="L58" s="4" t="inlineStr"/>
-      <c r="M58" s="4" t="inlineStr"/>
-      <c r="N58" s="4" t="inlineStr"/>
+      <c r="H58" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>系统组成章：前/后面板布局（指示灯/串口/心跳口/扩展插槽/电源）；接口高级信息区分电口/光口（光口不支持修改双工，速率10/100/1000M自适应）</t>
+        </is>
+      </c>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>接口体系：物理/子接口/AE聚合/HA/解密镜像/旁接/集群以太网/蜂窝（SIM双卡）多类型；接口速度10/100Mbps可选</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>待查资料（规格项）：G96：25G/40G/2.5G/5G接口速率与国产型号需查产品目录→V清单</t>
+        </is>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t>[R55→主证据矩阵#96] 天融信CHM:系统组成[topic32]+配置接口高级信息[ref487722465]；PA:webhelp p332-341/p428，admin p477</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -2985,7 +4241,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>待评估（原表备注：涉及硬件，等待研究院的评估结论）</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -2993,13 +4249,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr"/>
-      <c r="I59" s="5" t="inlineStr"/>
-      <c r="J59" s="5" t="inlineStr"/>
-      <c r="K59" s="5" t="inlineStr"/>
-      <c r="L59" s="5" t="inlineStr"/>
-      <c r="M59" s="5" t="inlineStr"/>
-      <c r="N59" s="5" t="inlineStr"/>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>系统组成章：前/后面板布局（指示灯/串口/心跳口/扩展插槽/电源）；接口高级信息区分电口/光口（光口不支持修改双工，速率10/100/1000M自适应）</t>
+        </is>
+      </c>
+      <c r="J59" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>接口体系：物理/子接口/AE聚合/HA/解密镜像/旁接/集群以太网/蜂窝（SIM双卡）多类型；接口速度10/100Mbps可选</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>PA优势·TS待实测：G96：PA收发器监控（show transceiver光衰）有据；TS光衰查看待实测→V清单</t>
+        </is>
+      </c>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>[R56→主证据矩阵#96] 天融信CHM:系统组成[topic32]+配置接口高级信息[ref487722465]；PA:webhelp p332-341/p428，admin p477</t>
+        </is>
+      </c>
+      <c r="N59" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3029,7 +4313,7 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>待评估</t>
+          <t>待评估（原表备注：已提交研究院接口需求，等待研究院答复）</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -3037,13 +4321,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H60" s="4" t="inlineStr"/>
-      <c r="I60" s="4" t="inlineStr"/>
-      <c r="J60" s="4" t="inlineStr"/>
-      <c r="K60" s="4" t="inlineStr"/>
-      <c r="L60" s="4" t="inlineStr"/>
-      <c r="M60" s="4" t="inlineStr"/>
-      <c r="N60" s="4" t="inlineStr"/>
+      <c r="H60" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>DPD（对端失效检测：启用/间隔/超时时间，默认启用）；链路备份（接口级）；策略路由智能选路（负载均衡+链路备份）；HA+链路探测+BFD</t>
+        </is>
+      </c>
+      <c r="J60" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>Tunnel Monitor 隧道监控（失败故障转移至备份网关）；静态路由 Path Monitoring（ICMP探测）；IKEv1 失效对等检测</t>
+        </is>
+      </c>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>仅命名不同：E77：TS DPD+链路备份+策略路由/PA Tunnel Monitor+Path Monitoring；切换时间待实测</t>
+        </is>
+      </c>
+      <c r="M60" s="4" t="inlineStr">
+        <is>
+          <t>[R57→主证据矩阵#77] 天融信CHM:静态隧道[topic4]+链路备份[toc462834587]+高可用[toc462834581]；PA:webhelp p439/admin p1168</t>
+        </is>
+      </c>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -3077,13 +4389,41 @@
           <t>产品线</t>
         </is>
       </c>
-      <c r="H61" s="5" t="inlineStr"/>
-      <c r="I61" s="5" t="inlineStr"/>
-      <c r="J61" s="5" t="inlineStr"/>
-      <c r="K61" s="5" t="inlineStr"/>
-      <c r="L61" s="5" t="inlineStr"/>
-      <c r="M61" s="5" t="inlineStr"/>
-      <c r="N61" s="5" t="inlineStr"/>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>部分支持</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>SSL卸载策略（解密后送安全引擎检测）；“解密流量镜像到外部接口”专用功能未见手册说明——待验证（R58）</t>
+        </is>
+      </c>
+      <c r="J61" s="12" t="inlineStr">
+        <is>
+          <t>完全支持</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>解密镜像接口（Decryption Port Mirroring）：解密后流量镜像到专用接口供 IDS/抓包；需激活免费许可证</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>PA优势：B124：PA解密镜像接口+许可证完全支持；TS部分支持（解密排除有据，镜像输出待实测）</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="inlineStr">
+        <is>
+          <t>[R58→主证据矩阵#124] PA:webhelp p312 解密镜像接口+admin p1114</t>
+        </is>
+      </c>
+      <c r="N61" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3091,12 +4431,11 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -11910,12 +13249,11 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -15387,12 +16725,11 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -16438,12 +17775,11 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -16723,12 +18059,11 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -18613,6 +19948,5 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>